<commit_message>
Ya estan agregados todos los bancos en un solo archivo
</commit_message>
<xml_diff>
--- a/Reportes_banco/reporte banco normalizado.xlsx
+++ b/Reportes_banco/reporte banco normalizado.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Mi unidad\Modelo de automatizaciones\Dashboards\dashboards\Reportes_banco\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\Modelo de automatizaciones\Dashboards\dashboards\Reportes_banco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2EE9157-01FD-4008-A832-01D809CFB39A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{094713B9-F8A3-4569-8E80-5B6A61D46E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,29 +16,12 @@
     <sheet name="TABLA GENERAL - Egresos" sheetId="1" r:id="rId1"/>
     <sheet name="TABLA GENERAL - Ingresos" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TABLA GENERAL - Egresos'!$A$1:$J$118</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TABLA GENERAL - Ingresos'!$A$1:$I$46</definedName>
-  </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="195">
   <si>
     <t>BANCO</t>
   </si>
@@ -187,6 +170,9 @@
     <t>SAN JUAN</t>
   </si>
   <si>
+    <t>06/03/2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">IMPUESTO CREDITO LEY 25413 -  </t>
   </si>
   <si>
@@ -199,15 +185,192 @@
     <t>IMPUESTO CREDITO LEY 25413 - VAR-MARIO FERNANDO PASCUA</t>
   </si>
   <si>
+    <t>06/02/2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">IMPUESTO DEBITO LEY 25413 -  </t>
   </si>
   <si>
     <t xml:space="preserve">CHEQUE CLEARING CAMARA -  </t>
   </si>
   <si>
+    <t>06/01/2026</t>
+  </si>
+  <si>
     <t>DB TRANS INM BSJ.EMP - VAR-ITALA S.A.</t>
   </si>
   <si>
+    <t>ICBC</t>
+  </si>
+  <si>
+    <t>IMP S/DEB CT</t>
+  </si>
+  <si>
+    <t>IVA RG 2408</t>
+  </si>
+  <si>
+    <t>I V A</t>
+  </si>
+  <si>
+    <t>COM MANT CT</t>
+  </si>
+  <si>
+    <t>MERCADO PAGO</t>
+  </si>
+  <si>
+    <t>161951138580</t>
+  </si>
+  <si>
+    <t>release</t>
+  </si>
+  <si>
+    <t>161162668429</t>
+  </si>
+  <si>
+    <t>161165786359</t>
+  </si>
+  <si>
+    <t>162014833932</t>
+  </si>
+  <si>
+    <t>161222135473</t>
+  </si>
+  <si>
+    <t>161222355267</t>
+  </si>
+  <si>
+    <t>161222891259</t>
+  </si>
+  <si>
+    <t>161223370367</t>
+  </si>
+  <si>
+    <t>161223738275</t>
+  </si>
+  <si>
+    <t>161224152121</t>
+  </si>
+  <si>
+    <t>162018061966</t>
+  </si>
+  <si>
+    <t>161224750001</t>
+  </si>
+  <si>
+    <t>161225266641</t>
+  </si>
+  <si>
+    <t>162019067394</t>
+  </si>
+  <si>
+    <t>162136593502</t>
+  </si>
+  <si>
+    <t>161343826405</t>
+  </si>
+  <si>
+    <t>162159832188</t>
+  </si>
+  <si>
+    <t>161367245025</t>
+  </si>
+  <si>
+    <t>162178283156</t>
+  </si>
+  <si>
+    <t>161389946927</t>
+  </si>
+  <si>
+    <t>162187363796</t>
+  </si>
+  <si>
+    <t>161406196619</t>
+  </si>
+  <si>
+    <t>161406691149</t>
+  </si>
+  <si>
+    <t>162337016546</t>
+  </si>
+  <si>
+    <t>162336929786</t>
+  </si>
+  <si>
+    <t>162337047466</t>
+  </si>
+  <si>
+    <t>161540134057</t>
+  </si>
+  <si>
+    <t>161551348743</t>
+  </si>
+  <si>
+    <t>161560368041</t>
+  </si>
+  <si>
+    <t>FRANCES</t>
+  </si>
+  <si>
+    <t>IMPUESTO LEY 02/06/26 00005</t>
+  </si>
+  <si>
+    <t>LEY NRO 25.4 01/06/26 00004</t>
+  </si>
+  <si>
+    <t>COMISION MOV 05/26 181981860</t>
+  </si>
+  <si>
+    <t>IVA TASA GRA</t>
+  </si>
+  <si>
+    <t>PERCEPCION I</t>
+  </si>
+  <si>
+    <t>COM.MANT.PQ  05/26 181981860</t>
+  </si>
+  <si>
+    <t>LEY NRO 25.4 29/05/26 00002</t>
+  </si>
+  <si>
+    <t>SUPERVIELLE</t>
+  </si>
+  <si>
+    <t>18/05/2026</t>
+  </si>
+  <si>
+    <t>Impuesto Débitos y Créditos/DB</t>
+  </si>
+  <si>
+    <t>IVA</t>
+  </si>
+  <si>
+    <t>OPERACIÓN 0 GENERADA EL 18/05/26</t>
+  </si>
+  <si>
+    <t>COMIS.TRANSFERENCIAS</t>
+  </si>
+  <si>
+    <t>Transferencia por CBU</t>
+  </si>
+  <si>
+    <t>CONCEPTO: Transferencia enviada TERMINAL: TESP0000 CBU: 0070112520000039502982 DOCUMENTO: 30708645326 NOMBRE: ITALA S.A.</t>
+  </si>
+  <si>
+    <t>15/05/2026</t>
+  </si>
+  <si>
+    <t>Impuesto Débitos y Créditos/CR</t>
+  </si>
+  <si>
+    <t>12/05/2026</t>
+  </si>
+  <si>
+    <t>OPERACIÓN 0 GENERADA EL 12/05/26</t>
+  </si>
+  <si>
+    <t>11/05/2026</t>
+  </si>
+  <si>
     <t>INGRESOS</t>
   </si>
   <si>
@@ -311,6 +474,138 @@
   </si>
   <si>
     <t>CR POR DEBIN - VAR-ITALA S A</t>
+  </si>
+  <si>
+    <t>161953208056</t>
+  </si>
+  <si>
+    <t>161162832875</t>
+  </si>
+  <si>
+    <t>161166420989</t>
+  </si>
+  <si>
+    <t>161168139265</t>
+  </si>
+  <si>
+    <t>161987204586</t>
+  </si>
+  <si>
+    <t>161994709840</t>
+  </si>
+  <si>
+    <t>159300440406</t>
+  </si>
+  <si>
+    <t>159305848896</t>
+  </si>
+  <si>
+    <t>162018820398</t>
+  </si>
+  <si>
+    <t>161232668531</t>
+  </si>
+  <si>
+    <t>159395095748</t>
+  </si>
+  <si>
+    <t>159400793932</t>
+  </si>
+  <si>
+    <t>159400761272</t>
+  </si>
+  <si>
+    <t>162154752182</t>
+  </si>
+  <si>
+    <t>158662693493</t>
+  </si>
+  <si>
+    <t>161373920691</t>
+  </si>
+  <si>
+    <t>161374895787</t>
+  </si>
+  <si>
+    <t>161377540255</t>
+  </si>
+  <si>
+    <t>158687238279</t>
+  </si>
+  <si>
+    <t>158687590809</t>
+  </si>
+  <si>
+    <t>162208740884</t>
+  </si>
+  <si>
+    <t>159567285016</t>
+  </si>
+  <si>
+    <t>159573292000</t>
+  </si>
+  <si>
+    <t>158800667543</t>
+  </si>
+  <si>
+    <t>162305959324</t>
+  </si>
+  <si>
+    <t>158801614705</t>
+  </si>
+  <si>
+    <t>162368154656</t>
+  </si>
+  <si>
+    <t>161571563917</t>
+  </si>
+  <si>
+    <t>161650782577</t>
+  </si>
+  <si>
+    <t>TRANSF.BANEL 27247950082</t>
+  </si>
+  <si>
+    <t>CTE 27247950082</t>
+  </si>
+  <si>
+    <t>TRANSF.BANEL 27438393507</t>
+  </si>
+  <si>
+    <t>CTE 27438393507</t>
+  </si>
+  <si>
+    <t>TRANSF.BANEL 20465438283</t>
+  </si>
+  <si>
+    <t>CTE 20465438283</t>
+  </si>
+  <si>
+    <t>TRF  IN COEL 20366079832</t>
+  </si>
+  <si>
+    <t>CTE 000011110008</t>
+  </si>
+  <si>
+    <t>DNET CREDITO NE4091657</t>
+  </si>
+  <si>
+    <t>CTE 091657       072-00000946135        ITALA S.A.</t>
+  </si>
+  <si>
+    <t>TRF  IN COEL 30708645326</t>
+  </si>
+  <si>
+    <t>CTE 000000000008</t>
+  </si>
+  <si>
+    <t>TRF  IN COEL 23149808469</t>
+  </si>
+  <si>
+    <t>Crédito por Transferencia</t>
+  </si>
+  <si>
+    <t>CONCEPTO: Transferencia recibida TERMINAL: MBSP0001 NOMBRE: AZARA PAMELA JHOANA DOCUMENTO: 27330585973 LETINI: A</t>
   </si>
 </sst>
 </file>
@@ -366,12 +661,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -674,16 +968,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J118"/>
+  <dimension ref="A1:J172"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="19.08984375" customWidth="1"/>
-    <col min="4" max="4" width="19.36328125" customWidth="1"/>
-    <col min="5" max="5" width="12.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.08984375" customWidth="1"/>
-    <col min="7" max="7" width="16.36328125" customWidth="1"/>
-    <col min="9" max="9" width="14.6328125" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" customWidth="1"/>
+    <col min="5" max="5" width="20.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -2509,12 +2797,12 @@
         <v>48</v>
       </c>
       <c r="B109" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C109" t="s">
-        <v>49</v>
-      </c>
-      <c r="E109" s="2">
+        <v>50</v>
+      </c>
+      <c r="E109">
         <v>18000</v>
       </c>
     </row>
@@ -2523,12 +2811,12 @@
         <v>48</v>
       </c>
       <c r="B110" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C110" t="s">
-        <v>49</v>
-      </c>
-      <c r="E110" s="2">
+        <v>50</v>
+      </c>
+      <c r="E110">
         <v>54000</v>
       </c>
     </row>
@@ -2537,12 +2825,12 @@
         <v>48</v>
       </c>
       <c r="B111" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C111" t="s">
-        <v>50</v>
-      </c>
-      <c r="E111" s="2">
+        <v>51</v>
+      </c>
+      <c r="E111">
         <v>26906017.100000001</v>
       </c>
     </row>
@@ -2551,12 +2839,12 @@
         <v>48</v>
       </c>
       <c r="B112" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C112" t="s">
-        <v>51</v>
-      </c>
-      <c r="E112" s="2">
+        <v>52</v>
+      </c>
+      <c r="E112">
         <v>161436.1</v>
       </c>
     </row>
@@ -2565,12 +2853,12 @@
         <v>48</v>
       </c>
       <c r="B113" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C113" t="s">
-        <v>52</v>
-      </c>
-      <c r="E113" s="2">
+        <v>53</v>
+      </c>
+      <c r="E113">
         <v>24270</v>
       </c>
     </row>
@@ -2579,12 +2867,12 @@
         <v>48</v>
       </c>
       <c r="B114" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C114" t="s">
-        <v>49</v>
-      </c>
-      <c r="E114" s="2">
+        <v>50</v>
+      </c>
+      <c r="E114">
         <v>9707.1299999999992</v>
       </c>
     </row>
@@ -2593,12 +2881,12 @@
         <v>48</v>
       </c>
       <c r="B115" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="C115" t="s">
-        <v>49</v>
-      </c>
-      <c r="E115" s="2">
+        <v>50</v>
+      </c>
+      <c r="E115">
         <v>1615.01</v>
       </c>
     </row>
@@ -2607,12 +2895,12 @@
         <v>48</v>
       </c>
       <c r="B116" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="C116" t="s">
-        <v>53</v>
-      </c>
-      <c r="E116" s="2">
+        <v>55</v>
+      </c>
+      <c r="E116">
         <v>3429</v>
       </c>
     </row>
@@ -2621,12 +2909,12 @@
         <v>48</v>
       </c>
       <c r="B117" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="C117" t="s">
-        <v>54</v>
-      </c>
-      <c r="E117" s="2">
+        <v>56</v>
+      </c>
+      <c r="E117">
         <v>571500</v>
       </c>
     </row>
@@ -2635,27 +2923,888 @@
         <v>48</v>
       </c>
       <c r="B118" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="C118" t="s">
-        <v>55</v>
-      </c>
-      <c r="E118" s="2">
+        <v>58</v>
+      </c>
+      <c r="E118">
         <v>1900000</v>
       </c>
     </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>59</v>
+      </c>
+      <c r="B119" t="s">
+        <v>16</v>
+      </c>
+      <c r="C119" t="s">
+        <v>60</v>
+      </c>
+      <c r="E119">
+        <v>319.92</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
+        <v>59</v>
+      </c>
+      <c r="B120" t="s">
+        <v>17</v>
+      </c>
+      <c r="C120" t="s">
+        <v>61</v>
+      </c>
+      <c r="E120">
+        <v>1290</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
+        <v>59</v>
+      </c>
+      <c r="B121" t="s">
+        <v>17</v>
+      </c>
+      <c r="C121" t="s">
+        <v>62</v>
+      </c>
+      <c r="E121">
+        <v>9030</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
+        <v>59</v>
+      </c>
+      <c r="B122" t="s">
+        <v>17</v>
+      </c>
+      <c r="C122" t="s">
+        <v>63</v>
+      </c>
+      <c r="E122">
+        <v>43000</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
+        <v>64</v>
+      </c>
+      <c r="B123" t="s">
+        <v>17</v>
+      </c>
+      <c r="C123" t="s">
+        <v>65</v>
+      </c>
+      <c r="D123" t="s">
+        <v>66</v>
+      </c>
+      <c r="E123">
+        <v>452700</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
+        <v>64</v>
+      </c>
+      <c r="B124" t="s">
+        <v>17</v>
+      </c>
+      <c r="C124" t="s">
+        <v>67</v>
+      </c>
+      <c r="D124" t="s">
+        <v>66</v>
+      </c>
+      <c r="E124">
+        <v>3400000</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
+        <v>64</v>
+      </c>
+      <c r="B125" t="s">
+        <v>17</v>
+      </c>
+      <c r="C125" t="s">
+        <v>68</v>
+      </c>
+      <c r="D125" t="s">
+        <v>66</v>
+      </c>
+      <c r="E125">
+        <v>201200</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
+        <v>64</v>
+      </c>
+      <c r="B126" t="s">
+        <v>17</v>
+      </c>
+      <c r="C126" t="s">
+        <v>69</v>
+      </c>
+      <c r="D126" t="s">
+        <v>66</v>
+      </c>
+      <c r="E126">
+        <v>150900</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
+        <v>64</v>
+      </c>
+      <c r="B127" t="s">
+        <v>17</v>
+      </c>
+      <c r="C127" t="s">
+        <v>70</v>
+      </c>
+      <c r="D127" t="s">
+        <v>66</v>
+      </c>
+      <c r="E127">
+        <v>452700</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
+        <v>64</v>
+      </c>
+      <c r="B128" t="s">
+        <v>17</v>
+      </c>
+      <c r="C128" t="s">
+        <v>71</v>
+      </c>
+      <c r="D128" t="s">
+        <v>66</v>
+      </c>
+      <c r="E128">
+        <v>321555.93</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
+        <v>64</v>
+      </c>
+      <c r="B129" t="s">
+        <v>17</v>
+      </c>
+      <c r="C129" t="s">
+        <v>72</v>
+      </c>
+      <c r="D129" t="s">
+        <v>66</v>
+      </c>
+      <c r="E129">
+        <v>311121.65000000002</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
+        <v>64</v>
+      </c>
+      <c r="B130" t="s">
+        <v>17</v>
+      </c>
+      <c r="C130" t="s">
+        <v>73</v>
+      </c>
+      <c r="D130" t="s">
+        <v>66</v>
+      </c>
+      <c r="E130">
+        <v>501372.02</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
+        <v>64</v>
+      </c>
+      <c r="B131" t="s">
+        <v>17</v>
+      </c>
+      <c r="C131" t="s">
+        <v>74</v>
+      </c>
+      <c r="D131" t="s">
+        <v>66</v>
+      </c>
+      <c r="E131">
+        <v>490221.78</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
+        <v>64</v>
+      </c>
+      <c r="B132" t="s">
+        <v>17</v>
+      </c>
+      <c r="C132" t="s">
+        <v>75</v>
+      </c>
+      <c r="D132" t="s">
+        <v>66</v>
+      </c>
+      <c r="E132">
+        <v>474257.09</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
+        <v>64</v>
+      </c>
+      <c r="B133" t="s">
+        <v>17</v>
+      </c>
+      <c r="C133" t="s">
+        <v>76</v>
+      </c>
+      <c r="D133" t="s">
+        <v>66</v>
+      </c>
+      <c r="E133">
+        <v>459934.3</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
+        <v>64</v>
+      </c>
+      <c r="B134" t="s">
+        <v>17</v>
+      </c>
+      <c r="C134" t="s">
+        <v>77</v>
+      </c>
+      <c r="D134" t="s">
+        <v>66</v>
+      </c>
+      <c r="E134">
+        <v>613667.32999999996</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
+        <v>64</v>
+      </c>
+      <c r="B135" t="s">
+        <v>17</v>
+      </c>
+      <c r="C135" t="s">
+        <v>78</v>
+      </c>
+      <c r="D135" t="s">
+        <v>66</v>
+      </c>
+      <c r="E135">
+        <v>598118.82999999996</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A136" t="s">
+        <v>64</v>
+      </c>
+      <c r="B136" t="s">
+        <v>17</v>
+      </c>
+      <c r="C136" t="s">
+        <v>79</v>
+      </c>
+      <c r="D136" t="s">
+        <v>66</v>
+      </c>
+      <c r="E136">
+        <v>591515.71</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
+        <v>64</v>
+      </c>
+      <c r="B137" t="s">
+        <v>16</v>
+      </c>
+      <c r="C137" t="s">
+        <v>80</v>
+      </c>
+      <c r="D137" t="s">
+        <v>66</v>
+      </c>
+      <c r="E137">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
+        <v>64</v>
+      </c>
+      <c r="B138" t="s">
+        <v>16</v>
+      </c>
+      <c r="C138" t="s">
+        <v>81</v>
+      </c>
+      <c r="D138" t="s">
+        <v>66</v>
+      </c>
+      <c r="E138">
+        <v>1056300</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A139" t="s">
+        <v>64</v>
+      </c>
+      <c r="B139" t="s">
+        <v>16</v>
+      </c>
+      <c r="C139" t="s">
+        <v>82</v>
+      </c>
+      <c r="D139" t="s">
+        <v>66</v>
+      </c>
+      <c r="E139">
+        <v>503000</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
+        <v>64</v>
+      </c>
+      <c r="B140" t="s">
+        <v>16</v>
+      </c>
+      <c r="C140" t="s">
+        <v>83</v>
+      </c>
+      <c r="D140" t="s">
+        <v>66</v>
+      </c>
+      <c r="E140">
+        <v>30180</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
+        <v>64</v>
+      </c>
+      <c r="B141" t="s">
+        <v>16</v>
+      </c>
+      <c r="C141" t="s">
+        <v>84</v>
+      </c>
+      <c r="D141" t="s">
+        <v>66</v>
+      </c>
+      <c r="E141">
+        <v>2069342</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
+        <v>64</v>
+      </c>
+      <c r="B142" t="s">
+        <v>16</v>
+      </c>
+      <c r="C142" t="s">
+        <v>85</v>
+      </c>
+      <c r="D142" t="s">
+        <v>66</v>
+      </c>
+      <c r="E142">
+        <v>20309.29</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
+        <v>64</v>
+      </c>
+      <c r="B143" t="s">
+        <v>16</v>
+      </c>
+      <c r="C143" t="s">
+        <v>86</v>
+      </c>
+      <c r="D143" t="s">
+        <v>66</v>
+      </c>
+      <c r="E143">
+        <v>466652.17</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
+        <v>64</v>
+      </c>
+      <c r="B144" t="s">
+        <v>16</v>
+      </c>
+      <c r="C144" t="s">
+        <v>87</v>
+      </c>
+      <c r="D144" t="s">
+        <v>66</v>
+      </c>
+      <c r="E144">
+        <v>1100000</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
+        <v>64</v>
+      </c>
+      <c r="B145" t="s">
+        <v>16</v>
+      </c>
+      <c r="C145" t="s">
+        <v>88</v>
+      </c>
+      <c r="D145" t="s">
+        <v>66</v>
+      </c>
+      <c r="E145">
+        <v>8800000</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
+        <v>64</v>
+      </c>
+      <c r="B146" t="s">
+        <v>11</v>
+      </c>
+      <c r="C146" t="s">
+        <v>89</v>
+      </c>
+      <c r="D146" t="s">
+        <v>66</v>
+      </c>
+      <c r="E146">
+        <v>312606.45</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
+        <v>64</v>
+      </c>
+      <c r="B147" t="s">
+        <v>11</v>
+      </c>
+      <c r="C147" t="s">
+        <v>90</v>
+      </c>
+      <c r="D147" t="s">
+        <v>66</v>
+      </c>
+      <c r="E147">
+        <v>142094.46</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
+        <v>64</v>
+      </c>
+      <c r="B148" t="s">
+        <v>11</v>
+      </c>
+      <c r="C148" t="s">
+        <v>91</v>
+      </c>
+      <c r="D148" t="s">
+        <v>66</v>
+      </c>
+      <c r="E148">
+        <v>142094.46</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
+        <v>64</v>
+      </c>
+      <c r="B149" t="s">
+        <v>11</v>
+      </c>
+      <c r="C149" t="s">
+        <v>92</v>
+      </c>
+      <c r="D149" t="s">
+        <v>66</v>
+      </c>
+      <c r="E149">
+        <v>168543.2</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>64</v>
+      </c>
+      <c r="B150" t="s">
+        <v>11</v>
+      </c>
+      <c r="C150" t="s">
+        <v>93</v>
+      </c>
+      <c r="D150" t="s">
+        <v>66</v>
+      </c>
+      <c r="E150">
+        <v>100600</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
+        <v>64</v>
+      </c>
+      <c r="B151" t="s">
+        <v>11</v>
+      </c>
+      <c r="C151" t="s">
+        <v>94</v>
+      </c>
+      <c r="D151" t="s">
+        <v>66</v>
+      </c>
+      <c r="E151">
+        <v>43113.37</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
+        <v>95</v>
+      </c>
+      <c r="B152" t="s">
+        <v>11</v>
+      </c>
+      <c r="C152" t="s">
+        <v>96</v>
+      </c>
+      <c r="E152">
+        <v>842.2</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A153" t="s">
+        <v>95</v>
+      </c>
+      <c r="B153" t="s">
+        <v>16</v>
+      </c>
+      <c r="C153" t="s">
+        <v>97</v>
+      </c>
+      <c r="E153">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A154" t="s">
+        <v>95</v>
+      </c>
+      <c r="B154" t="s">
+        <v>16</v>
+      </c>
+      <c r="C154" t="s">
+        <v>98</v>
+      </c>
+      <c r="E154">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A155" t="s">
+        <v>95</v>
+      </c>
+      <c r="B155" t="s">
+        <v>16</v>
+      </c>
+      <c r="C155" t="s">
+        <v>99</v>
+      </c>
+      <c r="E155">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A156" t="s">
+        <v>95</v>
+      </c>
+      <c r="B156" t="s">
+        <v>16</v>
+      </c>
+      <c r="C156" t="s">
+        <v>100</v>
+      </c>
+      <c r="E156">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A157" t="s">
+        <v>95</v>
+      </c>
+      <c r="B157" t="s">
+        <v>16</v>
+      </c>
+      <c r="C157" t="s">
+        <v>101</v>
+      </c>
+      <c r="E157">
+        <v>111200</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A158" t="s">
+        <v>95</v>
+      </c>
+      <c r="B158" t="s">
+        <v>16</v>
+      </c>
+      <c r="C158" t="s">
+        <v>99</v>
+      </c>
+      <c r="E158">
+        <v>23352</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A159" t="s">
+        <v>95</v>
+      </c>
+      <c r="B159" t="s">
+        <v>16</v>
+      </c>
+      <c r="C159" t="s">
+        <v>100</v>
+      </c>
+      <c r="E159">
+        <v>3336</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A160" t="s">
+        <v>95</v>
+      </c>
+      <c r="B160" t="s">
+        <v>17</v>
+      </c>
+      <c r="C160" t="s">
+        <v>102</v>
+      </c>
+      <c r="E160">
+        <v>10267.799999999999</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A161" t="s">
+        <v>103</v>
+      </c>
+      <c r="B161" t="s">
+        <v>104</v>
+      </c>
+      <c r="C161" t="s">
+        <v>105</v>
+      </c>
+      <c r="E161">
+        <v>3.78</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A162" t="s">
+        <v>103</v>
+      </c>
+      <c r="B162" t="s">
+        <v>104</v>
+      </c>
+      <c r="C162" t="s">
+        <v>105</v>
+      </c>
+      <c r="E162">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A163" t="s">
+        <v>103</v>
+      </c>
+      <c r="B163" t="s">
+        <v>104</v>
+      </c>
+      <c r="C163" t="s">
+        <v>106</v>
+      </c>
+      <c r="D163" t="s">
+        <v>107</v>
+      </c>
+      <c r="E163">
+        <v>132.30000000000001</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A164" t="s">
+        <v>103</v>
+      </c>
+      <c r="B164" t="s">
+        <v>104</v>
+      </c>
+      <c r="C164" t="s">
+        <v>108</v>
+      </c>
+      <c r="D164" t="s">
+        <v>107</v>
+      </c>
+      <c r="E164">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A165" t="s">
+        <v>103</v>
+      </c>
+      <c r="B165" t="s">
+        <v>104</v>
+      </c>
+      <c r="C165" t="s">
+        <v>109</v>
+      </c>
+      <c r="D165" t="s">
+        <v>110</v>
+      </c>
+      <c r="E165">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A166" t="s">
+        <v>103</v>
+      </c>
+      <c r="B166" t="s">
+        <v>111</v>
+      </c>
+      <c r="C166" t="s">
+        <v>112</v>
+      </c>
+      <c r="E166">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A167" t="s">
+        <v>103</v>
+      </c>
+      <c r="B167" t="s">
+        <v>113</v>
+      </c>
+      <c r="C167" t="s">
+        <v>105</v>
+      </c>
+      <c r="E167">
+        <v>3.78</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A168" t="s">
+        <v>103</v>
+      </c>
+      <c r="B168" t="s">
+        <v>113</v>
+      </c>
+      <c r="C168" t="s">
+        <v>105</v>
+      </c>
+      <c r="E168">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A169" t="s">
+        <v>103</v>
+      </c>
+      <c r="B169" t="s">
+        <v>113</v>
+      </c>
+      <c r="C169" t="s">
+        <v>106</v>
+      </c>
+      <c r="D169" t="s">
+        <v>114</v>
+      </c>
+      <c r="E169">
+        <v>132.30000000000001</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A170" t="s">
+        <v>103</v>
+      </c>
+      <c r="B170" t="s">
+        <v>113</v>
+      </c>
+      <c r="C170" t="s">
+        <v>108</v>
+      </c>
+      <c r="D170" t="s">
+        <v>114</v>
+      </c>
+      <c r="E170">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A171" t="s">
+        <v>103</v>
+      </c>
+      <c r="B171" t="s">
+        <v>113</v>
+      </c>
+      <c r="C171" t="s">
+        <v>109</v>
+      </c>
+      <c r="D171" t="s">
+        <v>110</v>
+      </c>
+      <c r="E171">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A172" t="s">
+        <v>103</v>
+      </c>
+      <c r="B172" t="s">
+        <v>115</v>
+      </c>
+      <c r="C172" t="s">
+        <v>112</v>
+      </c>
+      <c r="E172">
+        <v>12000</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J118" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="5" width="13.6328125" customWidth="1"/>
+    <col min="2" max="2" width="25.26953125" customWidth="1"/>
+    <col min="3" max="3" width="23.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -2675,7 +3824,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>56</v>
+        <v>116</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
@@ -2684,7 +3833,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>57</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -2695,7 +3844,7 @@
         <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>118</v>
       </c>
       <c r="E2">
         <v>11000000</v>
@@ -2709,7 +3858,7 @@
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>119</v>
       </c>
       <c r="E3">
         <v>5681400</v>
@@ -2723,7 +3872,7 @@
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="E4">
         <v>27300000</v>
@@ -2737,7 +3886,7 @@
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>121</v>
       </c>
       <c r="E5">
         <v>3400000</v>
@@ -2751,10 +3900,10 @@
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>62</v>
+        <v>122</v>
       </c>
       <c r="D6" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E6">
         <v>132806.73000000001</v>
@@ -2768,10 +3917,10 @@
         <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>122</v>
       </c>
       <c r="D7" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E7">
         <v>730840.32</v>
@@ -2785,7 +3934,7 @@
         <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
+        <v>124</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
@@ -2802,7 +3951,7 @@
         <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>65</v>
+        <v>125</v>
       </c>
       <c r="D9" t="s">
         <v>22</v>
@@ -2819,7 +3968,7 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>66</v>
+        <v>126</v>
       </c>
       <c r="D10" t="s">
         <v>44</v>
@@ -2836,7 +3985,7 @@
         <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>127</v>
       </c>
       <c r="D11" t="s">
         <v>44</v>
@@ -2853,7 +4002,7 @@
         <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>128</v>
       </c>
       <c r="D12" t="s">
         <v>44</v>
@@ -2870,10 +4019,10 @@
         <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>122</v>
       </c>
       <c r="D13" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E13">
         <v>11973.75</v>
@@ -2887,10 +4036,10 @@
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>122</v>
       </c>
       <c r="D14" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E14">
         <v>1133798.3999999999</v>
@@ -2904,7 +4053,7 @@
         <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>69</v>
+        <v>129</v>
       </c>
       <c r="D15" t="s">
         <v>22</v>
@@ -2921,7 +4070,7 @@
         <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="D16" t="s">
         <v>22</v>
@@ -2938,7 +4087,7 @@
         <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="D17" t="s">
         <v>22</v>
@@ -2955,7 +4104,7 @@
         <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>71</v>
+        <v>131</v>
       </c>
       <c r="D18" t="s">
         <v>44</v>
@@ -2972,7 +4121,7 @@
         <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="D19" t="s">
         <v>44</v>
@@ -2989,7 +4138,7 @@
         <v>16</v>
       </c>
       <c r="C20" t="s">
-        <v>73</v>
+        <v>133</v>
       </c>
       <c r="D20" t="s">
         <v>44</v>
@@ -3006,7 +4155,7 @@
         <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>74</v>
+        <v>134</v>
       </c>
       <c r="D21" t="s">
         <v>44</v>
@@ -3023,10 +4172,10 @@
         <v>16</v>
       </c>
       <c r="C22" t="s">
-        <v>75</v>
+        <v>135</v>
       </c>
       <c r="D22" t="s">
-        <v>76</v>
+        <v>136</v>
       </c>
       <c r="E22">
         <v>432000</v>
@@ -3040,10 +4189,10 @@
         <v>11</v>
       </c>
       <c r="C23" t="s">
-        <v>62</v>
+        <v>122</v>
       </c>
       <c r="D23" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E23">
         <v>833112</v>
@@ -3057,7 +4206,7 @@
         <v>11</v>
       </c>
       <c r="C24" t="s">
-        <v>65</v>
+        <v>125</v>
       </c>
       <c r="D24" t="s">
         <v>22</v>
@@ -3071,13 +4220,13 @@
         <v>20</v>
       </c>
       <c r="B25" t="s">
-        <v>77</v>
+        <v>137</v>
       </c>
       <c r="C25" t="s">
-        <v>62</v>
+        <v>122</v>
       </c>
       <c r="D25" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E25">
         <v>164758.79999999999</v>
@@ -3088,13 +4237,13 @@
         <v>20</v>
       </c>
       <c r="B26" t="s">
-        <v>77</v>
+        <v>137</v>
       </c>
       <c r="C26" t="s">
-        <v>62</v>
+        <v>122</v>
       </c>
       <c r="D26" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E26">
         <v>1124854.3999999999</v>
@@ -3108,7 +4257,7 @@
         <v>17</v>
       </c>
       <c r="C27" t="s">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="D27" t="s">
         <v>22</v>
@@ -3125,10 +4274,10 @@
         <v>17</v>
       </c>
       <c r="C28" t="s">
-        <v>78</v>
+        <v>138</v>
       </c>
       <c r="D28" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E28">
         <v>4990000</v>
@@ -3142,10 +4291,10 @@
         <v>16</v>
       </c>
       <c r="C29" t="s">
-        <v>79</v>
+        <v>139</v>
       </c>
       <c r="D29" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E29">
         <v>21670000</v>
@@ -3159,10 +4308,10 @@
         <v>16</v>
       </c>
       <c r="C30" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="D30" t="s">
-        <v>76</v>
+        <v>136</v>
       </c>
       <c r="E30">
         <v>4000000</v>
@@ -3176,10 +4325,10 @@
         <v>11</v>
       </c>
       <c r="C31" t="s">
-        <v>79</v>
+        <v>139</v>
       </c>
       <c r="D31" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E31">
         <v>28720000</v>
@@ -3193,10 +4342,10 @@
         <v>11</v>
       </c>
       <c r="C32" t="s">
-        <v>79</v>
+        <v>139</v>
       </c>
       <c r="D32" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E32">
         <v>50000000</v>
@@ -3210,10 +4359,10 @@
         <v>11</v>
       </c>
       <c r="C33" t="s">
-        <v>79</v>
+        <v>139</v>
       </c>
       <c r="D33" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E33">
         <v>50000000</v>
@@ -3227,10 +4376,10 @@
         <v>11</v>
       </c>
       <c r="C34" t="s">
-        <v>79</v>
+        <v>139</v>
       </c>
       <c r="D34" t="s">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="E34">
         <v>18000000</v>
@@ -3244,7 +4393,7 @@
         <v>11</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>129</v>
       </c>
       <c r="D35" t="s">
         <v>22</v>
@@ -3261,7 +4410,7 @@
         <v>11</v>
       </c>
       <c r="C36" t="s">
-        <v>81</v>
+        <v>141</v>
       </c>
       <c r="D36" t="s">
         <v>44</v>
@@ -3278,7 +4427,7 @@
         <v>11</v>
       </c>
       <c r="C37" t="s">
-        <v>82</v>
+        <v>142</v>
       </c>
       <c r="D37" t="s">
         <v>44</v>
@@ -3295,7 +4444,7 @@
         <v>11</v>
       </c>
       <c r="C38" t="s">
-        <v>83</v>
+        <v>143</v>
       </c>
       <c r="D38" t="s">
         <v>44</v>
@@ -3312,7 +4461,7 @@
         <v>11</v>
       </c>
       <c r="C39" t="s">
-        <v>84</v>
+        <v>144</v>
       </c>
       <c r="D39" t="s">
         <v>28</v>
@@ -3326,12 +4475,12 @@
         <v>48</v>
       </c>
       <c r="B40" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C40" t="s">
-        <v>85</v>
-      </c>
-      <c r="E40" s="2">
+        <v>145</v>
+      </c>
+      <c r="E40">
         <v>9000000</v>
       </c>
     </row>
@@ -3340,12 +4489,12 @@
         <v>48</v>
       </c>
       <c r="B41" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C41" t="s">
-        <v>86</v>
-      </c>
-      <c r="E41" s="2">
+        <v>146</v>
+      </c>
+      <c r="E41">
         <v>3000000</v>
       </c>
     </row>
@@ -3354,12 +4503,12 @@
         <v>48</v>
       </c>
       <c r="B42" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C42" t="s">
-        <v>87</v>
-      </c>
-      <c r="E42" s="2">
+        <v>147</v>
+      </c>
+      <c r="E42">
         <v>9000000</v>
       </c>
     </row>
@@ -3368,12 +4517,12 @@
         <v>48</v>
       </c>
       <c r="B43" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C43" t="s">
-        <v>88</v>
-      </c>
-      <c r="E43" s="2">
+        <v>148</v>
+      </c>
+      <c r="E43">
         <v>4045000</v>
       </c>
     </row>
@@ -3382,12 +4531,12 @@
         <v>48</v>
       </c>
       <c r="B44" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="C44" t="s">
-        <v>89</v>
-      </c>
-      <c r="E44" s="2">
+        <v>149</v>
+      </c>
+      <c r="E44">
         <v>1617855.35</v>
       </c>
     </row>
@@ -3396,12 +4545,12 @@
         <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="C45" t="s">
-        <v>89</v>
-      </c>
-      <c r="E45" s="2">
+        <v>149</v>
+      </c>
+      <c r="E45">
         <v>269167.53999999998</v>
       </c>
     </row>
@@ -3410,17 +4559,662 @@
         <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="C46" t="s">
-        <v>90</v>
-      </c>
-      <c r="E46" s="2">
+        <v>150</v>
+      </c>
+      <c r="E46">
         <v>1000000</v>
       </c>
     </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>64</v>
+      </c>
+      <c r="B47" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" t="s">
+        <v>151</v>
+      </c>
+      <c r="D47" t="s">
+        <v>66</v>
+      </c>
+      <c r="E47">
+        <v>1988000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>64</v>
+      </c>
+      <c r="B48" t="s">
+        <v>17</v>
+      </c>
+      <c r="C48" t="s">
+        <v>152</v>
+      </c>
+      <c r="D48" t="s">
+        <v>66</v>
+      </c>
+      <c r="E48">
+        <v>1988000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>64</v>
+      </c>
+      <c r="B49" t="s">
+        <v>17</v>
+      </c>
+      <c r="C49" t="s">
+        <v>153</v>
+      </c>
+      <c r="D49" t="s">
+        <v>66</v>
+      </c>
+      <c r="E49">
+        <v>1491000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>64</v>
+      </c>
+      <c r="B50" t="s">
+        <v>17</v>
+      </c>
+      <c r="C50" t="s">
+        <v>154</v>
+      </c>
+      <c r="D50" t="s">
+        <v>66</v>
+      </c>
+      <c r="E50">
+        <v>410522</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>64</v>
+      </c>
+      <c r="B51" t="s">
+        <v>17</v>
+      </c>
+      <c r="C51" t="s">
+        <v>155</v>
+      </c>
+      <c r="D51" t="s">
+        <v>66</v>
+      </c>
+      <c r="E51">
+        <v>169974</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>64</v>
+      </c>
+      <c r="B52" t="s">
+        <v>17</v>
+      </c>
+      <c r="C52" t="s">
+        <v>156</v>
+      </c>
+      <c r="D52" t="s">
+        <v>66</v>
+      </c>
+      <c r="E52">
+        <v>397600</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>64</v>
+      </c>
+      <c r="B53" t="s">
+        <v>17</v>
+      </c>
+      <c r="C53" t="s">
+        <v>157</v>
+      </c>
+      <c r="D53" t="s">
+        <v>66</v>
+      </c>
+      <c r="E53">
+        <v>465075.5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>64</v>
+      </c>
+      <c r="B54" t="s">
+        <v>17</v>
+      </c>
+      <c r="C54" t="s">
+        <v>158</v>
+      </c>
+      <c r="D54" t="s">
+        <v>66</v>
+      </c>
+      <c r="E54">
+        <v>415848.03</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>64</v>
+      </c>
+      <c r="B55" t="s">
+        <v>17</v>
+      </c>
+      <c r="C55" t="s">
+        <v>159</v>
+      </c>
+      <c r="D55" t="s">
+        <v>66</v>
+      </c>
+      <c r="E55">
+        <v>574532</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>64</v>
+      </c>
+      <c r="B56" t="s">
+        <v>17</v>
+      </c>
+      <c r="C56" t="s">
+        <v>160</v>
+      </c>
+      <c r="D56" t="s">
+        <v>66</v>
+      </c>
+      <c r="E56">
+        <v>361145.05</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>64</v>
+      </c>
+      <c r="B57" t="s">
+        <v>16</v>
+      </c>
+      <c r="C57" t="s">
+        <v>161</v>
+      </c>
+      <c r="D57" t="s">
+        <v>66</v>
+      </c>
+      <c r="E57">
+        <v>368456.55</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>64</v>
+      </c>
+      <c r="B58" t="s">
+        <v>16</v>
+      </c>
+      <c r="C58" t="s">
+        <v>162</v>
+      </c>
+      <c r="D58" t="s">
+        <v>66</v>
+      </c>
+      <c r="E58">
+        <v>369239.52</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>64</v>
+      </c>
+      <c r="B59" t="s">
+        <v>16</v>
+      </c>
+      <c r="C59" t="s">
+        <v>163</v>
+      </c>
+      <c r="D59" t="s">
+        <v>66</v>
+      </c>
+      <c r="E59">
+        <v>369239.52</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>64</v>
+      </c>
+      <c r="B60" t="s">
+        <v>16</v>
+      </c>
+      <c r="C60" t="s">
+        <v>164</v>
+      </c>
+      <c r="D60" t="s">
+        <v>66</v>
+      </c>
+      <c r="E60">
+        <v>1988000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>64</v>
+      </c>
+      <c r="B61" t="s">
+        <v>16</v>
+      </c>
+      <c r="C61" t="s">
+        <v>165</v>
+      </c>
+      <c r="D61" t="s">
+        <v>66</v>
+      </c>
+      <c r="E61">
+        <v>465075.5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" t="s">
+        <v>16</v>
+      </c>
+      <c r="C62" t="s">
+        <v>166</v>
+      </c>
+      <c r="D62" t="s">
+        <v>66</v>
+      </c>
+      <c r="E62">
+        <v>8566292</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>64</v>
+      </c>
+      <c r="B63" t="s">
+        <v>16</v>
+      </c>
+      <c r="C63" t="s">
+        <v>167</v>
+      </c>
+      <c r="D63" t="s">
+        <v>66</v>
+      </c>
+      <c r="E63">
+        <v>135179.43</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>64</v>
+      </c>
+      <c r="B64" t="s">
+        <v>16</v>
+      </c>
+      <c r="C64" t="s">
+        <v>168</v>
+      </c>
+      <c r="D64" t="s">
+        <v>66</v>
+      </c>
+      <c r="E64">
+        <v>130214</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>16</v>
+      </c>
+      <c r="C65" t="s">
+        <v>169</v>
+      </c>
+      <c r="D65" t="s">
+        <v>66</v>
+      </c>
+      <c r="E65">
+        <v>79839.899999999994</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>64</v>
+      </c>
+      <c r="B66" t="s">
+        <v>16</v>
+      </c>
+      <c r="C66" t="s">
+        <v>170</v>
+      </c>
+      <c r="D66" t="s">
+        <v>66</v>
+      </c>
+      <c r="E66">
+        <v>604163.5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>64</v>
+      </c>
+      <c r="B67" t="s">
+        <v>16</v>
+      </c>
+      <c r="C67" t="s">
+        <v>171</v>
+      </c>
+      <c r="D67" t="s">
+        <v>66</v>
+      </c>
+      <c r="E67">
+        <v>91209.44</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>64</v>
+      </c>
+      <c r="B68" t="s">
+        <v>11</v>
+      </c>
+      <c r="C68" t="s">
+        <v>172</v>
+      </c>
+      <c r="D68" t="s">
+        <v>66</v>
+      </c>
+      <c r="E68">
+        <v>359020.9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>64</v>
+      </c>
+      <c r="B69" t="s">
+        <v>11</v>
+      </c>
+      <c r="C69" t="s">
+        <v>173</v>
+      </c>
+      <c r="D69" t="s">
+        <v>66</v>
+      </c>
+      <c r="E69">
+        <v>341895.69</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>64</v>
+      </c>
+      <c r="B70" t="s">
+        <v>11</v>
+      </c>
+      <c r="C70" t="s">
+        <v>174</v>
+      </c>
+      <c r="D70" t="s">
+        <v>66</v>
+      </c>
+      <c r="E70">
+        <v>139088</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>64</v>
+      </c>
+      <c r="B71" t="s">
+        <v>11</v>
+      </c>
+      <c r="C71" t="s">
+        <v>175</v>
+      </c>
+      <c r="D71" t="s">
+        <v>66</v>
+      </c>
+      <c r="E71">
+        <v>190185</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>64</v>
+      </c>
+      <c r="B72" t="s">
+        <v>11</v>
+      </c>
+      <c r="C72" t="s">
+        <v>176</v>
+      </c>
+      <c r="D72" t="s">
+        <v>66</v>
+      </c>
+      <c r="E72">
+        <v>186899.5</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>64</v>
+      </c>
+      <c r="B73" t="s">
+        <v>11</v>
+      </c>
+      <c r="C73" t="s">
+        <v>177</v>
+      </c>
+      <c r="D73" t="s">
+        <v>66</v>
+      </c>
+      <c r="E73">
+        <v>298200</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>64</v>
+      </c>
+      <c r="B74" t="s">
+        <v>11</v>
+      </c>
+      <c r="C74" t="s">
+        <v>178</v>
+      </c>
+      <c r="D74" t="s">
+        <v>66</v>
+      </c>
+      <c r="E74">
+        <v>22663.200000000001</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>64</v>
+      </c>
+      <c r="B75" t="s">
+        <v>137</v>
+      </c>
+      <c r="C75" t="s">
+        <v>179</v>
+      </c>
+      <c r="D75" t="s">
+        <v>66</v>
+      </c>
+      <c r="E75">
+        <v>497000</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>95</v>
+      </c>
+      <c r="B76" t="s">
+        <v>11</v>
+      </c>
+      <c r="C76" t="s">
+        <v>180</v>
+      </c>
+      <c r="D76" t="s">
+        <v>181</v>
+      </c>
+      <c r="E76">
+        <v>515000</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>95</v>
+      </c>
+      <c r="B77" t="s">
+        <v>11</v>
+      </c>
+      <c r="C77" t="s">
+        <v>182</v>
+      </c>
+      <c r="D77" t="s">
+        <v>183</v>
+      </c>
+      <c r="E77">
+        <v>955500</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>95</v>
+      </c>
+      <c r="B78" t="s">
+        <v>11</v>
+      </c>
+      <c r="C78" t="s">
+        <v>184</v>
+      </c>
+      <c r="D78" t="s">
+        <v>185</v>
+      </c>
+      <c r="E78">
+        <v>1198800</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>95</v>
+      </c>
+      <c r="B79" t="s">
+        <v>11</v>
+      </c>
+      <c r="C79" t="s">
+        <v>186</v>
+      </c>
+      <c r="D79" t="s">
+        <v>187</v>
+      </c>
+      <c r="E79">
+        <v>1984500</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>95</v>
+      </c>
+      <c r="B80" t="s">
+        <v>17</v>
+      </c>
+      <c r="C80" t="s">
+        <v>188</v>
+      </c>
+      <c r="D80" t="s">
+        <v>189</v>
+      </c>
+      <c r="E80">
+        <v>14500000</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>95</v>
+      </c>
+      <c r="B81" t="s">
+        <v>17</v>
+      </c>
+      <c r="C81" t="s">
+        <v>190</v>
+      </c>
+      <c r="D81" t="s">
+        <v>191</v>
+      </c>
+      <c r="E81">
+        <v>95000000</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>95</v>
+      </c>
+      <c r="B82" t="s">
+        <v>17</v>
+      </c>
+      <c r="C82" t="s">
+        <v>192</v>
+      </c>
+      <c r="D82" t="s">
+        <v>187</v>
+      </c>
+      <c r="E82">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>103</v>
+      </c>
+      <c r="B83" t="s">
+        <v>111</v>
+      </c>
+      <c r="C83" t="s">
+        <v>193</v>
+      </c>
+      <c r="D83" t="s">
+        <v>194</v>
+      </c>
+      <c r="E83">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>103</v>
+      </c>
+      <c r="B84" t="s">
+        <v>115</v>
+      </c>
+      <c r="C84" t="s">
+        <v>193</v>
+      </c>
+      <c r="D84" t="s">
+        <v>194</v>
+      </c>
+      <c r="E84">
+        <v>2000000</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I46" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>